<commit_message>
Refine fourth-week task breakdown and issue assignments
</commit_message>
<xml_diff>
--- a/docs/test-data/第三周课程清单导入合法测试数据.xlsx
+++ b/docs/test-data/第三周课程清单导入合法测试数据.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试数据" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="课程导入" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,22 +25,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001F2937"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8F0FE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -55,14 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,149 +413,125 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>所属专业代码</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>适用年级</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
         <is>
           <t>课程代码</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>课程名称</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>学分</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>080901</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>CS260</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>数字取证技术</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>TESTCS301</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>软件质量保证</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>080901</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>CS261</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>智能系统工程</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TESTCS302</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>专业认证导论</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>080902</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>SW204</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>软件过程度量</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>080701</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>EE304</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>嵌入式接口技术</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B4" t="n">
+        <v>2023</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TESTSE401</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>软件过程改进</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>